<commit_message>
Add the end-to-end sign-in and quotation email story to the workbook.
ONB-11 matches the new Jira story and includes the portal, Outlook code, and sample quotation data.
</commit_message>
<xml_diff>
--- a/docs/broker-onboarding-user-stories-login-with-code.xlsx
+++ b/docs/broker-onboarding-user-stories-login-with-code.xlsx
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1063,6 +1063,53 @@
         </is>
       </c>
     </row>
+    <row r="13" ht="120" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>ONB-11</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Sign in with the email code and email the quotation</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>As a broker, I want to sign in with the employee login and the Outlook verification code, then complete onboarding and email the quotation, so that one flow takes a customer from the portal to the sent quotation.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>The broker opens https://birlasoftfscdemo-dev-ed.develop.my.site.com/brokerportal/s/customer-search-portal, chooses Login, then Are you an employee? login here. The broker enters username jitendra.sonawane@birlasoft.com.fscdemo, clicks Log In, enters the portal password, and clicks Log In. Salesforce emails a verification code. On this machine, classic Outlook is open. The broker reads the newest message from noreply@salesforce.com whose subject contains Verify your identity in Salesforce, takes the digits on the Verification Code line, enters that code, and clicks Verify. The broker clicks Start Onboarding, searches for AJC BILLINGHAM, selects AJC BILLINGHAM LTD, and creates or updates the customer account. The broker enters test@test.com for CAMERON, Andrew David, marks that contact as the quote contact and the authorized signatory, and saves. On Loan Information the broker enters total premium 60000, deposit 9 percent, and gross rate 9, chooses 6 instalments and purpose Property Insurance, calculates, and continues. On Financial Information the broker chooses Experian, enters credit score 750, and saves. The broker creates a quote, opens it, sets disclose commission to Yes, and saves. The broker creates the PDF, clicks Save and Email Quote, confirms the message, and sends it to test@test.com.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>1. Given the broker is not signed in, when the broker opens https://birlasoftfscdemo-dev-ed.develop.my.site.com/brokerportal/s/customer-search-portal and chooses Login, then Are you an employee? login here is available.
+2. Given the employee login, when the broker enters username jitendra.sonawane@birlasoft.com.fscdemo and clicks Log In, then the broker can enter the portal password and click Log In.
+3. Given the password was submitted, when Salesforce emails a verification code, then classic Outlook on this machine has a new message from noreply@salesforce.com whose subject contains Verify your identity in Salesforce.
+4. Given that message, when the broker reads the digits on the Verification Code line, enters that code, and clicks Verify, then the welcome screen is shown.
+5. Given the welcome screen, when the broker clicks Start Onboarding, searches for AJC BILLINGHAM, and selects AJC BILLINGHAM LTD, status Active, address Surtees Business Park, Stockton-On-Tees, TS18 3HR, then the broker can create or update the customer account.
+6. Given the account is saved, when the broker enters test@test.com for CAMERON, Andrew David, marks that contact as the quote contact and the authorized signatory, and clicks Create or Update Contacts, then Loan Information opens.
+7. Given Loan Information, when the broker enters total premium 60000, deposit 9 percent, and gross rate 9, chooses 6 instalments and purpose Property Insurance, and clicks Calculate, then the calculated loan summary is shown.
+8. Given the loan summary, when the broker clicks Continue, chooses credit source Experian, enters credit score 750, and clicks Save, then the qualification record opens and shows that credit source and score.
+9. Given the qualification record, when the broker clicks Create Quote, opens the quote, sets disclose commission to Yes, and saves, then the broker commission is calculated and shown on the quote.
+10. Given the quote is saved, when the broker clicks Create PDF and then Save and Email Quote, confirms the message, and sends, then the quotation is emailed to test@test.com and remains on the quote.
+11. End-to-end use case: the broker opens the portal, chooses Login, clicks Are you an employee? login here, enters the username, clicks Log In, enters the portal password, clicks Log In, reads the verification code from the newest Salesforce email in Outlook, enters that code, clicks Verify, starts onboarding, saves AJC BILLINGHAM LTD and contact CAMERON, Andrew David, calculates the loan, saves Experian and credit score 750, creates the quote, saves disclose commission Yes, creates the PDF, and sends the quotation email to test@test.com.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Portal https://birlasoftfscdemo-dev-ed.develop.my.site.com/brokerportal/s/customer-search-portal. Username jitendra.sonawane@birlasoft.com.fscdemo. Password is the portal password for that username. Verification email from noreply@salesforce.com, subject Verify your identity in Salesforce, line Verification Code. Search AJC BILLINGHAM. Company AJC BILLINGHAM LTD. Status Active. Address Surtees Business Park, Stockton-On-Tees, TS18 3HR. Contact CAMERON, Andrew David. Email test@test.com. Premium 60000. Deposit 9 percent. Instalments 6. Gross rate 9. Purpose Property Insurance. Deposit amount 5400.00. Credit charge 4914.00. Monthly instalment 9919.00. Balance payable excluding deposit 59514.00. Net rate 7. Credit source Experian. Credit score 750. Disclose commission Yes. Commission percent 2.00. Commission amount 1092.00. Email To test@test.com.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1075,7 +1122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E70"/>
+  <dimension ref="A1:E81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2600,6 +2647,241 @@
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>ONB-11</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Sign in with the email code and email the quotation</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Given the broker is not signed in, when the broker opens https://birlasoftfscdemo-dev-ed.develop.my.site.com/brokerportal/s/customer-search-portal and chooses Login, then Are you an employee? login here is available.</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>Portal https://birlasoftfscdemo-dev-ed.develop.my.site.com/brokerportal/s/customer-search-portal. Username jitendra.sonawane@birlasoft.com.fscdemo. Password is the portal password for that username. Verification email from noreply@salesforce.com, subject Verify your identity in Salesforce, line Verification Code. Search AJC BILLINGHAM. Company AJC BILLINGHAM LTD. Status Active. Address Surtees Business Park, Stockton-On-Tees, TS18 3HR. Contact CAMERON, Andrew David. Email test@test.com. Premium 60000. Deposit 9 percent. Instalments 6. Gross rate 9. Purpose Property Insurance. Deposit amount 5400.00. Credit charge 4914.00. Monthly instalment 9919.00. Balance payable excluding deposit 59514.00. Net rate 7. Credit source Experian. Credit score 750. Disclose commission Yes. Commission percent 2.00. Commission amount 1092.00. Email To test@test.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>ONB-11</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Sign in with the email code and email the quotation</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Given the employee login, when the broker enters username jitendra.sonawane@birlasoft.com.fscdemo and clicks Log In, then the broker can enter the portal password and click Log In.</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>ONB-11</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Sign in with the email code and email the quotation</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Given the password was submitted, when Salesforce emails a verification code, then classic Outlook on this machine has a new message from noreply@salesforce.com whose subject contains Verify your identity in Salesforce.</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>ONB-11</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Sign in with the email code and email the quotation</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Given that message, when the broker reads the digits on the Verification Code line, enters that code, and clicks Verify, then the welcome screen is shown.</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>ONB-11</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Sign in with the email code and email the quotation</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Given the welcome screen, when the broker clicks Start Onboarding, searches for AJC BILLINGHAM, and selects AJC BILLINGHAM LTD, status Active, address Surtees Business Park, Stockton-On-Tees, TS18 3HR, then the broker can create or update the customer account.</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>ONB-11</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Sign in with the email code and email the quotation</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Given the account is saved, when the broker enters test@test.com for CAMERON, Andrew David, marks that contact as the quote contact and the authorized signatory, and clicks Create or Update Contacts, then Loan Information opens.</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>ONB-11</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Sign in with the email code and email the quotation</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Given Loan Information, when the broker enters total premium 60000, deposit 9 percent, and gross rate 9, chooses 6 instalments and purpose Property Insurance, and clicks Calculate, then the calculated loan summary is shown.</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>ONB-11</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Sign in with the email code and email the quotation</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Given the loan summary, when the broker clicks Continue, chooses credit source Experian, enters credit score 750, and clicks Save, then the qualification record opens and shows that credit source and score.</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>ONB-11</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Sign in with the email code and email the quotation</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Given the qualification record, when the broker clicks Create Quote, opens the quote, sets disclose commission to Yes, and saves, then the broker commission is calculated and shown on the quote.</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>ONB-11</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Sign in with the email code and email the quotation</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Given the quote is saved, when the broker clicks Create PDF and then Save and Email Quote, confirms the message, and sends, then the quotation is emailed to test@test.com and remains on the quote.</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>ONB-11</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Sign in with the email code and email the quotation</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>End-to-end use case: the broker opens the portal, chooses Login, clicks Are you an employee? login here, enters the username, clicks Log In, enters the portal password, clicks Log In, reads the verification code from the newest Salesforce email in Outlook, enters that code, clicks Verify, starts onboarding, saves AJC BILLINGHAM LTD and contact CAMERON, Andrew David, calculates the loan, saves Experian and credit score 750, creates the quote, saves disclose commission Yes, creates the PDF, and sends the quotation email to test@test.com.</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>
@@ -2613,7 +2895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3379,6 +3661,600 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Portal URL</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>https://birlasoftfscdemo-dev-ed.develop.my.site.com/brokerportal/s/customer-search-portal</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Address opened for this story</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Yes. Another portal environment still follows the story.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Username</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>jitendra.sonawane@birlasoft.com.fscdemo</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Username entered after the employee login</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Password</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Portal password for that username</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Entered after the first Log In. Not copied into this sheet.</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Verification mail from</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>noreply@salesforce.com</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Sender of the code email in Outlook</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Verification mail subject</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Verify your identity in Salesforce</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Subject text used to find the newest message</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Verification code line</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Verification Code</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Line in the message that holds the digits</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>The digits change on every sign-in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Company search</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>AJC BILLINGHAM</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Text typed into search</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Company name</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>AJC BILLINGHAM LTD</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Company selected</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Status on the selected company</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Surtees Business Park, Stockton-On-Tees, TS18 3HR</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Address on the selected company</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>CAMERON, Andrew David</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Quote contact and authorized signatory</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>test@test.com</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Contact email and quotation email To</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Total premium</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>60000</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Amount the broker enters</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Deposit percent</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Amount the broker enters</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>No. of repayments</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>One choice from 3, 6, 9, 12, 24</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>The allowed list is the rule. 6 is the sample.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Gross rate</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Amount the broker enters</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Purpose of loan</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Property Insurance</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>One choice from Property Insurance, Life Insurance, Medical insurance</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>The allowed list is the rule. This purpose is the sample.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Credit source</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Experian</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>One choice from Experian, Equifax, TransUnion</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>The allowed list is the rule. Experian is the sample.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Credit score</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>750</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Score the broker enters</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Disclose commission</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Selected, then the quote is saved</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Commission percent</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Calculated after save</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>C end to end</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Commission amount</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>1092.00</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Calculated after save and printed when disclosure is on</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>